<commit_message>
feat: add audio system and data databases
</commit_message>
<xml_diff>
--- a/UPDATE_LOG.xlsx
+++ b/UPDATE_LOG.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,26 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>버전</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>날짜</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>담당자</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>수정 내용</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -454,15 +474,547 @@
           <t>0.1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>프로젝트 시작</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>상세 기획 명세서 8개 작성 (GDD, 경제, 성장, UI 스펙 등)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>프로젝트 상세 기획 단계 시작</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>v0.2.0 기획 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>인게임 핵심 루프 MVP 구현 완료 (타이틀, 메인, 튜토리얼, 손님 시스템, 주방 제조, 평가 정산)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>버전 관리 적용 및 dev 브랜치 이관</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>v0.3.0 MVP 마일스톤 달성</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0.3.1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>코드 의존성 진단 보고서 작성</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Resources.Load 의존성 분석 및 Sprite 직접 참조 전환 계획 수립</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>런타임 최적화 분석</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>타이틀 화면 나무 질감 UI 버튼 및 프리미엄 배경 이미지 적용, 이름 입력 모달창 레이아웃 가로 정렬</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TitleScreenUIBuilder 비주얼 개편</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TitleScreenManager 클릭 이벤트(OnStartClicked, OnSettingsClicked) private -&gt; public 변경 및 OnEnable/OnDisable 리스너 활성화하여 인스펙터 노출 버그 해결</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>UI/UX 고도화 및 버그 픽스</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0.4.1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>5인의 손님 캐릭터 스프라이트 실연결 및 preserveAspect 비율 유지 처리</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CustomerAppearanceUIBuilder 손님 렌더링 최적화</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>손님 비주얼 개선</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>메인 테마 BGM 사운드 디자인 명세서 (SOUND_DESIGN_DOCUMENT.md) 작성</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>사운드 기획 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0.5.1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>한국 테마 (Korea Theme BGM) 사운드 디자인 명세서 추가</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>사운드 기획 갱신</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0.5.2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>중국 테마 (China Theme BGM) 사운드 디자인 명세서 추가</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>사운드 기획 갱신</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0.5.3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>일본 테마 (Japan Theme BGM) 사운드 디자인 명세서 추가</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>사운드 기획 갱신</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>0.5.4</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>베트남 테마 (Vietnam Theme BGM) 사운드 디자인 명세서 추가</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>사운드 기획 갱신</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>0.5.5</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>키르기스스탄 테마 (Kyrgyzstan Theme BGM) 사운드 디자인 명세서 추가</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>사운드 기획 갱신</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Created SFX Design Specification</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>SFX 기획 신규 작성</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Created AUDIO_IMPLEMENTATION_GUIDE.md and expanded SFX doc</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Unity 오디오 구현 가이드 신규 작성</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>v0.8</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Phase 1 구현: AudioManager 확장 (CrossFade, Ambience, AudioMixer 연동) 및 SettingsManager 업데이트</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>v0.9</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Phase 2 구현: SFX Object Pool 추가, Polyphony 동시 재생 제어, Pitch/Volume 랜덤화 및 Priority 속성을 위한 SfxDatabase 도입</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Phase 3 구현: ThemeAudioData 및 ThemeDatabase 도입, SettingsManager 하드코딩(switch문) 제거, 데이터 기반 국가 테마 구조 확립</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>v1.1</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>최종 개선 적용: AudioManager.Awake()에서 SfxDatabase 및 ThemeDatabase의 Pre-warming 적용으로 첫 재생 지연(Hitch) 방지</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>v1.2</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>문서 통합: 사운드 기획, 효과음 기획, 기술 구현 문서를 단일 마스터 문서(AUDIO_MASTER_DOCUMENT.md)로 통합 및 중복 내용 제거</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>DrinkDatabase 시스템 구현: DrinkData(SO), DrinkDatabase(SO), SetupDrinkDatabase(Editor Tool) 추가. CountryType enum, 5종 초기 음료 자동 생성, OnEnable() 안전 초기화.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>v1.3.1</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>SetupDrinkDatabase 정책 변경: InitializeOnLoad 자동 실행 제거. Tools &gt; Setup &gt; Create Drink Database 수동 실행 방식으로 전환. Idempotent 보장 (기존 에셋 보존, 없는 항목만 생성).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>v1.3.2</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>AI_DEVELOPMENT_RULES.md 수정 (v1.2): 셋업 툴의 에셋 수정/덮어쓰기 금지 및 변경이 필요할 경우 별도의 Tools &gt; Migration 또는 Upgrade 기능으로 분리 명시.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>v1.4.0</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>IngredientDatabase 시스템 구현: IngredientData(SO), IngredientDatabase(SO), SetupIngredientDatabase(Editor Setup Tool) 추가. 공통 자원 설계 적용(국가 정보 제외), Shyr Chai를 포함한 7종 재료 에셋 멱등 셋업 지원.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>v1.5.0</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>RecipeDatabase 시스템 구현: RecipeData(SO), RecipeDatabase(SO), SetupRecipeDatabase(Editor Setup Tool) 추가. recipeId/우림 조건 제외, targetDrink 1:1 + IngredientRequirement 1:N 설계. 기존 DrinkDatabase/IngredientDatabase 무수정, Shyr Chai 포함 5종 레시피 자동 링킹, Idempotent 보장.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: snapshot current project state
</commit_message>
<xml_diff>
--- a/UPDATE_LOG.xlsx
+++ b/UPDATE_LOG.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,11 +474,19 @@
           <t>0.1</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>프로젝트 시작</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -501,11 +509,16 @@
           <t>프로젝트 상세 기획 단계 시작</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>v0.2.0 기획 완료</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -528,11 +541,16 @@
           <t>버전 관리 적용 및 dev 브랜치 이관</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>v0.3.0 MVP 마일스톤 달성</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -555,11 +573,16 @@
           <t>Resources.Load 의존성 분석 및 Sprite 직접 참조 전환 계획 수립</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>런타임 최적화 분석</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -592,6 +615,10 @@
           <t>UI/UX 고도화 및 버그 픽스</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -614,11 +641,16 @@
           <t>CustomerAppearanceUIBuilder 손님 렌더링 최적화</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>손님 비주얼 개선</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -636,11 +668,17 @@
           <t>메인 테마 BGM 사운드 디자인 명세서 (SOUND_DESIGN_DOCUMENT.md) 작성</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>사운드 기획 추가</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -658,11 +696,17 @@
           <t>한국 테마 (Korea Theme BGM) 사운드 디자인 명세서 추가</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>사운드 기획 갱신</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -680,11 +724,17 @@
           <t>중국 테마 (China Theme BGM) 사운드 디자인 명세서 추가</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>사운드 기획 갱신</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -702,11 +752,17 @@
           <t>일본 테마 (Japan Theme BGM) 사운드 디자인 명세서 추가</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>사운드 기획 갱신</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -724,11 +780,17 @@
           <t>베트남 테마 (Vietnam Theme BGM) 사운드 디자인 명세서 추가</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>사운드 기획 갱신</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -746,11 +808,17 @@
           <t>키르기스스탄 테마 (Kyrgyzstan Theme BGM) 사운드 디자인 명세서 추가</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>사운드 기획 갱신</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -768,11 +836,17 @@
           <t>Created SFX Design Specification</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>SFX 기획 신규 작성</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -790,13 +864,25 @@
           <t>Created AUDIO_IMPLEMENTATION_GUIDE.md and expanded SFX doc</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>Unity 오디오 구현 가이드 신규 작성</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>v0.8</t>
@@ -819,6 +905,12 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>v0.9</t>
@@ -841,6 +933,12 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>v1.0</t>
@@ -863,6 +961,12 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>v1.1</t>
@@ -885,6 +989,12 @@
       </c>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>v1.2</t>
@@ -907,6 +1017,12 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>v1.3</t>
@@ -929,6 +1045,12 @@
       </c>
     </row>
     <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>v1.3.1</t>
@@ -951,6 +1073,12 @@
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>v1.3.2</t>
@@ -973,6 +1101,12 @@
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>v1.4.0</t>
@@ -995,6 +1129,12 @@
       </c>
     </row>
     <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>v1.5.0</t>
@@ -1013,6 +1153,1210 @@
       <c r="J25" t="inlineStr">
         <is>
           <t>RecipeDatabase 시스템 구현: RecipeData(SO), RecipeDatabase(SO), SetupRecipeDatabase(Editor Setup Tool) 추가. recipeId/우림 조건 제외, targetDrink 1:1 + IngredientRequirement 1:N 설계. 기존 DrinkDatabase/IngredientDatabase 무수정, Shyr Chai 포함 5종 레시피 자동 링킹, Idempotent 보장.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>v1.6.0</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Brewing 시스템 확장(BrewingManager.cs): DrinkDatabase/RecipeDatabase SerializeField 추가(Inspector 연결), CanBrew(out string) 레시피 검증 API 추가, StartBrewingWithValidation() 신규 추가. 기존 Public API 시그니처 전체 보존. ConsumeIngredients/TODO Hook 미추가.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>v1.7.0</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Inventory 시스템 구현(v1.7.0): InventoryManager.cs 싱글톤 추가, Add/Consume/Get/HasEnough API 구현, GetSaveData/LoadSaveData 세이브 연동 API 설계(자체 저장배제 및 데이터 제공 전용), BrewingManager.CanBrew()에 재고 검증 루프 연동.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>v1.8.0</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Shop 시스템 구현(v1.8.0): ShopManager.cs 싱글톤 추가, GetAvailableIngredients/BuyIngredient API 구현, PlayerDataManager 직접 의존성 차단 및 CheckAndConsumeMoney(TODO) 연동, IsShopOpen 기본값 false 설정, unlockLevel 조건 배제.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>v1.9.0</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Money 시스템 구현(v1.9.0): MoneyManager.cs 싱글톤 추가, CurrentMoney(private set), startingMoney 인스펙터 지원, AddMoney/SpendMoney/CanAfford API 구현, ShopManager.CheckAndConsumeMoney() 실제 차감 연동. PlayerDataManager 수정 없음.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>v1.10.0</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>DayManager 시스템 구현(v1.10.0): DayManager.cs 싱글톤 추가. 하루 상태(Ready, Operating, Settlement) 관리, ShopManager 오픈/마감 연동, RecordSale/RecordCustomerServed 통계 기록, 정산 시 자동 저장 훅(TriggerAutoSave) 제공. MoneyManager 직접 조작 배제 및 비즈니스 규칙 반영.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>v1.11.0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>SaveManager 시스템 구현(v1.11.0): SaveManager.cs 싱글톤 추가. 유일한 저장/로드 관리자, GameSaveData 최상위 구조체 구현, SaveGame/LoadGame/HasSave/DeleteSave API 구현, SaveVersion 마이그레이션 대비 검사 및 TODO 반영, SAVE_KEY 상수화, DayManager 영업 결산 시 자동 저장 연동.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>v1.12.0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>CustomerManager &amp; CustomerDatabase 구현(v1.12.0): CustomerData 확장(displayNameKey/descriptionKey/nationality/portrait/sprite), CustomerDatabase(SO) 구축, CustomerManager 개편(Instantiate 배제, pure CustomerData Queue 관리), NotifyCustomerReady/OnCustomerArrived 훅 연동, DayManager Operating 조건 검사.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>v1.13.0</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>OrderManager &amp; OrderData 구현(v1.13.0): OrderData 클래스 추가 (orderId 단순 카운트), OrderManager 싱글톤 추가, CustomerManager.OnCustomerArrived 이벤트 연동, CompleteOrder(string brewedDrinkId) 검증, SelectDrinkForCustomer 확장구조 설계, DrinkDatabase Inspector 참조.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>v1.14.0</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>CustomerView 구현(v1.14.0): CustomerView.cs 클래스 추가 (UI Image 기반 노출/숨김), CustomerManager 이벤트 직접 구독 배제(외부 명시적 호출), Instantiate/Destroy 미사용(풀링 대비), ShowCustomer/HideCustomer/HasVisibleCustomer API 및 명시적 애니메이션 Hook 구현.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>v1.15.0</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>ServingManager 구현(v1.15.0): ServingManager.cs 싱글톤 추가 (서빙 흐름 제어 오케스트레이터), CustomerView 직접 참조 배제 및 OnServeSucceeded/OnServeFailed 이벤트 발생, OrderManager 검증 후 MoneyManager/DayManager/CustomerManager 순차 호출, OrderData 기반 최종 보상 금액 보관 확장 대비 TODO 작성.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>v1.16.0</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>AffinityManager 구현(v1.16.0): AffinityManager.cs 싱글톤 추가 (손님별 친밀도 수치 저장/조회 전담), ServingManager.OnServeSucceeded(customerId, drinkId, price) 시그니처 변경 및 전달받은 customerId로 친밀도 +1 간접 연동, SaveManager.cs에 AffinitySaveData 통합 세이브/로드 연결.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>v1.17.0</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>UnlockManager 구현(v1.17.0): UnlockConstants.cs (DEFAULT_UNLOCKED_IDS) 생성, UnlockManager.cs 싱글톤 추가 (Unlock, Lock, IsUnlocked, GetAllUnlockedIds API), InitializeDefaultUnlocks() 명시적 새 게임 API 분리 (Awake 자동호출 배제), SaveManager.cs에 UnlockSaveData 통합 세이브/로드 연결.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>v1.18.0</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>FurnitureManager 구현(v1.18.0): FurnitureManager.cs 싱글톤 추가, FurnitureStateChangeType enum 및 OnFurnitureStateChanged 이벤트 구현, PlaceFurniture() 자동 Active 부여 배제, LoadSaveData() 시 active ⊂ placed ⊂ owned 데이터 무결성 검증, SaveManager.cs에 FurnitureSaveData 통합 세이브/로드 연결.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>v1.20.0</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>SettingsManager 시스템 구현: 언어, BGM, SFX 볼륨 관리 및 통합 저장소 연동(SaveManager/LocalizationManager 수정)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>v1.21.0</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>UI Localization System 구현: LocalizedText 컴포넌트 추가로 자동 다국어 갱신 지원</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>v1.22.0</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>AudioManager 리팩토링: SettingsManager 연동 및 하위 호환성 유지(Wrapper API 적용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>v1.23.0</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>MainMenu 시스템(View/Controller) 분리 구현 및 이벤트 연동</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>v1.24.0</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Settings UI 시스템(MVP 패턴) 구현 및 Language/Volume 제어 분리 연동</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>v1.25.0</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>HUD 시스템 구현 (MVP 패턴 적용, Manager 이벤트 구독 연동)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>v1.26.0</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Brewing UI 시스템(MVP 패턴) 구현 및 BrewingManager 진행도 이벤트 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>v1.27.0</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Inventory UI 시스템(MVP 패턴) 구현 및 IngredientData localizationKey 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>v1.28.0</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Shop UI 시스템(MVP 패턴) 구현 및 ShopManager CanPurchase API 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>v1.29.0</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Furniture UI 시스템(MVP 패턴) 구현 및 FurnitureManager 배치 검증 API 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>v1.30.0</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Tutorial 시스템(MVP 패턴) 구현 및 TutorialHighlightRegistry/SaveManager 연동</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>v1.31.0</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Notification(Toast) 시스템(MVP 패턴) 구현 및 NotificationDisplayData/Controller 출력 코루틴 구축</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>v1.32.0</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Confirmation Dialog 시스템(MVP 패턴) 구현 및 DialogResult/CurrentDialog/ESC 연동</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>v1.33.0</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Scene Transition &amp; Loading 시스템(MVP 패턴) 구현 및 RequestTransition/ResetView/0~1 정규화 조율</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>v1.34.0</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Debug Panel 시스템(MVP 패턴) 구현 및 DebugCommand switch 처리/빌드 격리 전처리기 적용</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>v1.34.1</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>컴파일 에러전수 조치/기록(ERROR_RESOLVED_LOG) 및 파편 문서/스크립트 통폐합 정돈</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>v1.35.0</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Integration Phase 유니티 씬/오케스트레이션 셋업(SetupIntegrationScenes) 및 Smoke Test 가이드 구축</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>v1.36.0</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Gameplay Vertical Slice 통합 검증, 인스펙터 널 방어막 구축 및 이벤트 파라미터 유실 버그 수정</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>v1.36.1</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>자동 복구 구문 전면 제거 및 Fail Fast(Debug.LogError) 적용, 정적 검토/Play Mode 검증 구분 정리</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>v1.37.0</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>콘텐츠 제작(재료8종, 음료8종, 레시피8종, 손님5종) 및 초/중/후반 경제/진행 밸런스 구축</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>v1.38.0</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Content Expansion(재료22, 음료32, 레시피32, 손님20, 가구20, 해금35) 및 ContentValidator 에디터 툴 구축</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>v1.39.0</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>20일 플레이 테스트 검증 수행, 인플레이션/초반지루함 원인 분석 및 재료/음료 수치 튜닝</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>v1.40.0</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Production Phase Task #1: 첫 플레이(FTUE) 경험 개선, 씬 Fade 연출, SFX/Toast 피드백 및 튜토리얼 텍스트 튜닝</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>v1.41.0</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Production Phase Task #2: Juice 강화(Elastic Scale Pop 팝업/Toast 연출, 상점 구매/실패 SFX/Toast 피드백)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>v1.42.0</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Production Phase Task #3: RC 15대 필수 항목 QA 전수 검증 및 잔여 버그 0개 수렴 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>v1.43.0</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>콘솔 붉은 에러 100% 원인 추적 및 디버깅 (MainMenuController 메서드 복구, ShopController Notification 시그니처 튜닝)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>v1.44.0</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>유니티 콘솔 24개 CS1061 컴파일 에러 전수 추적 및 ScriptableObject 필드명 100% 매칭 수정</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>v1.45.0</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>사용자 보고 버그 수정: 튜토리얼 다음/건너뛰기 버튼 클릭 불능 해결 (TutorialController, TutorialView)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>v1.46.0</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>사용자 직접 리포트 3대 버그 수정 (튜토리얼 클릭 블로킹 해제, 시작하기 1회 튕김 수정, 설정 버튼 UI 연결)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>v1.46.0</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>AI Assistant</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>사용자 리포트 버그 C# 수정 시도 및 Play Mode 미검증/미해결 상태 기록 갱신</t>
         </is>
       </c>
     </row>

</xml_diff>